<commit_message>
feat(import): format Excel 10 cột + multi-shop + Nhóm menu
Cấu trúc mới: A=SĐT | B=Cat1 | C=Cat2 | D=Cat3 | E=Nhóm menu |
F=Tên | G=Mô tả | H=Giá | I=Size | J=Topping. SĐT đọc từng dòng
thay vì dòng đầu file — một file có thể chứa nhiều quán khác nhau.
saveImportMenu group theo SĐT → lưu đúng shop. Template cập nhật
dropdown 12 danh mục chuẩn ở cột B/C/D.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/template_nhap_menu_giao_nhanh.xlsx
+++ b/public/template_nhap_menu_giao_nhanh.xlsx
@@ -5,6 +5,7 @@
   <sheets>
     <sheet name="📋 Danh sách món" sheetId="1" r:id="rId1"/>
     <sheet name="📖 Hướng dẫn" sheetId="2" r:id="rId2"/>
+    <sheet name="_list" sheetId="3" r:id="rId3"/>
   </sheets>
 </workbook>
 </file>
@@ -398,132 +399,225 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L5"/>
+  <dimension ref="A1:J6"/>
   <cols>
-    <col min="1" max="1" width="22.83203125" customWidth="1"/>
-    <col min="2" max="2" width="16.83203125" customWidth="1"/>
-    <col min="3" max="3" width="26.83203125" customWidth="1"/>
-    <col min="4" max="4" width="32.83203125" customWidth="1"/>
-    <col min="5" max="5" width="14.83203125" customWidth="1"/>
-    <col min="6" max="6" width="18.83203125" customWidth="1"/>
-    <col min="7" max="7" width="12.83203125" customWidth="1"/>
-    <col min="8" max="8" width="10.83203125" customWidth="1"/>
-    <col min="9" max="9" width="10.83203125" customWidth="1"/>
-    <col min="10" max="10" width="10.83203125" customWidth="1"/>
-    <col min="11" max="11" width="20.83203125" customWidth="1"/>
-    <col min="12" max="12" width="24.83203125" customWidth="1"/>
+    <col min="1" max="1" width="14.83203125" customWidth="1"/>
+    <col min="2" max="2" width="20.83203125" customWidth="1"/>
+    <col min="3" max="3" width="20.83203125" customWidth="1"/>
+    <col min="4" max="4" width="20.83203125" customWidth="1"/>
+    <col min="5" max="5" width="16.83203125" customWidth="1"/>
+    <col min="6" max="6" width="28.83203125" customWidth="1"/>
+    <col min="7" max="7" width="34.83203125" customWidth="1"/>
+    <col min="8" max="8" width="14.83203125" customWidth="1"/>
+    <col min="9" max="9" width="30.83203125" customWidth="1"/>
+    <col min="10" max="10" width="36.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>SĐT_QUAN:</v>
+        <v>SĐT Quán *</v>
       </c>
       <c r="B1" t="str">
-        <v>0901234567 (điền SĐT cửa hàng vào đây)</v>
+        <v>Danh mục 1 *</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Danh mục 2</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Danh mục 3</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Nhóm menu</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Tên Món *</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Mô Tả</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Giá Bán * (đ)</v>
+      </c>
+      <c r="I1" t="str">
+        <v>Size và Giá (VD: M:0, L:5000)</v>
+      </c>
+      <c r="J1" t="str">
+        <v>Topping và Giá (VD: Trân châu:5000)</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Danh mục (tối đa 3)</v>
+        <v>0901234567</v>
       </c>
       <c r="B2" t="str">
-        <v>Nhóm menu</v>
+        <v>Cà phê - Trà sữa</v>
       </c>
       <c r="C2" t="str">
-        <v>Tên món</v>
+        <v/>
       </c>
       <c r="D2" t="str">
-        <v>Mô tả / Nguyên liệu</v>
+        <v/>
       </c>
       <c r="E2" t="str">
-        <v>Giá bán (đ)</v>
+        <v>Cà phê</v>
       </c>
       <c r="F2" t="str">
-        <v>Giá khuyến mãi (đ)</v>
+        <v>Cà phê đen đá</v>
       </c>
       <c r="G2" t="str">
-        <v>Badge</v>
-      </c>
-      <c r="H2" t="str">
-        <v>Đang bán</v>
+        <v>Cà phê phin truyền thống</v>
+      </c>
+      <c r="H2">
+        <v>17000</v>
       </c>
       <c r="I2" t="str">
-        <v>Giờ bán từ</v>
+        <v/>
       </c>
       <c r="J2" t="str">
-        <v>Giờ bán đến</v>
-      </c>
-      <c r="K2" t="str">
-        <v>Sizes</v>
-      </c>
-      <c r="L2" t="str">
-        <v>Toppings</v>
+        <v/>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Nước uống, Buổi sáng, Buổi trưa</v>
+        <v>0901234567</v>
       </c>
       <c r="B3" t="str">
+        <v>Cà phê - Trà sữa</v>
+      </c>
+      <c r="C3" t="str">
+        <v/>
+      </c>
+      <c r="D3" t="str">
+        <v/>
+      </c>
+      <c r="E3" t="str">
         <v>Cà phê</v>
       </c>
-      <c r="C3" t="str">
-        <v>Cà phê đen đá</v>
-      </c>
-      <c r="E3">
+      <c r="F3" t="str">
+        <v>Cà phê sữa đá</v>
+      </c>
+      <c r="G3" t="str">
+        <v/>
+      </c>
+      <c r="H3">
         <v>17000</v>
       </c>
-      <c r="H3" t="str">
-        <v>CÓ</v>
+      <c r="I3" t="str">
+        <v/>
+      </c>
+      <c r="J3" t="str">
+        <v/>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Nước uống, Buổi sáng, Buổi trưa</v>
+        <v>0901234567</v>
       </c>
       <c r="B4" t="str">
-        <v>Cà phê</v>
+        <v>Cà phê - Trà sữa</v>
       </c>
       <c r="C4" t="str">
-        <v>Cà phê sữa đá</v>
-      </c>
-      <c r="E4">
-        <v>17000</v>
-      </c>
-      <c r="H4" t="str">
-        <v>CÓ</v>
+        <v/>
+      </c>
+      <c r="D4" t="str">
+        <v/>
+      </c>
+      <c r="E4" t="str">
+        <v>Trà sữa</v>
+      </c>
+      <c r="F4" t="str">
+        <v>Trà sữa khoai môn</v>
+      </c>
+      <c r="G4" t="str">
+        <v>Béo thơm</v>
+      </c>
+      <c r="H4">
+        <v>35000</v>
+      </c>
+      <c r="I4" t="str">
+        <v>Nhỏ:0, Lớn:5000</v>
+      </c>
+      <c r="J4" t="str">
+        <v>Trân châu:5000, Thạch:5000</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Nước uống, Buổi sáng, Buổi trưa</v>
+        <v>0901234567</v>
       </c>
       <c r="B5" t="str">
-        <v>Cà phê</v>
+        <v>Cơm - Cơm hộp</v>
       </c>
       <c r="C5" t="str">
-        <v>Bạc xỉu</v>
-      </c>
-      <c r="E5">
-        <v>23000</v>
-      </c>
-      <c r="H5" t="str">
-        <v>CÓ</v>
+        <v>Ăn vặt - Vỉa hè</v>
+      </c>
+      <c r="D5" t="str">
+        <v/>
+      </c>
+      <c r="E5" t="str">
+        <v>Cơm trưa</v>
+      </c>
+      <c r="F5" t="str">
+        <v>Cơm sườn bì chả</v>
+      </c>
+      <c r="G5" t="str">
+        <v>Cơm + sườn + bì + chả</v>
+      </c>
+      <c r="H5">
+        <v>45000</v>
+      </c>
+      <c r="I5" t="str">
+        <v/>
+      </c>
+      <c r="J5" t="str">
+        <v>Trứng ốp:5000</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>0901234567</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Bún - Phở - Mì</v>
+      </c>
+      <c r="C6" t="str">
+        <v/>
+      </c>
+      <c r="D6" t="str">
+        <v/>
+      </c>
+      <c r="E6" t="str">
+        <v>Bún</v>
+      </c>
+      <c r="F6" t="str">
+        <v>Bún bò Huế</v>
+      </c>
+      <c r="G6" t="str">
+        <v>Bún bò đặc biệt</v>
+      </c>
+      <c r="H6">
+        <v>35000</v>
+      </c>
+      <c r="I6" t="str">
+        <v>Nhỏ:0, Lớn:10000</v>
+      </c>
+      <c r="J6" t="str">
+        <v>Giò heo:15000, Huyết:5000</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J6"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B22"/>
+  <dimension ref="A1:B26"/>
   <cols>
     <col min="1" max="1" width="14.83203125" customWidth="1"/>
-    <col min="2" max="2" width="70.83203125" customWidth="1"/>
+    <col min="2" max="2" width="72.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -533,151 +627,240 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>⭐ QUAN TRỌNG</v>
-      </c>
-      <c r="B3" t="str">
-        <v>Dòng đầu tiên (SĐT_QUAN:) là khóa nhận diện cửa hàng — BẮT BUỘC điền đúng SĐT</v>
+        <v>⭐ QUY TẮC QUAN TRỌNG</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>•</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Cột A (SĐT Quán) phải điền ở MỌI dòng — hệ thống dùng để tìm đúng quán</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>🔶 BƯỚC 1</v>
+        <v>•</v>
       </c>
       <c r="B5" t="str">
-        <v>Điền SĐT cửa hàng vào ô B1 (cạnh chữ SĐT_QUAN:)</v>
+        <v>Một file có thể chứa nhiều quán khác nhau (SĐT khác nhau ở cột A)</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>🔶 BƯỚC 2</v>
+        <v>•</v>
       </c>
       <c r="B6" t="str">
-        <v>Xóa các dòng mẫu (từ dòng 3 trở đi) → điền món của cửa hàng</v>
+        <v>Cột có dấu * là bắt buộc</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>🔶 CỘT A</v>
+      </c>
+      <c r="B8" t="str">
+        <v>SĐT Quán — lặp lại ở mỗi dòng. VD: 0901234567</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>🔶 CỘT B</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Danh mục 1 (bắt buộc) — chọn từ dropdown 12 danh mục chuẩn</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>🔶 CỘT C</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Danh mục 2 (tuỳ chọn) — để trống nếu không cần</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>🔶 CỘT D</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Danh mục 3 (tuỳ chọn) — để trống nếu không cần</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>🔶 CỘT E</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Nhóm menu — nhóm nội bộ hiển thị trong trang quán. VD: Cà phê, Trà sữa, Cơm trưa</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>🔶 CỘT F</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Tên món (bắt buộc)</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>🔶 CỘT G</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Mô tả / Nguyên liệu</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>🔶 CỘT H</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Giá bán (số nguyên VNĐ, bắt buộc). VD: 35000</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>🔶 CỘT I</v>
+      </c>
+      <c r="B16" t="str">
+        <v>Size và giá — định dạng: TênSize:GiáTăngThêm  VD: M:0, L:5000, XL:10000</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>🔶 CỘT J</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Topping và giá — định dạng: TênTopping:Giá  VD: Trân châu:5000, Thạch:5000</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>📌 DANH MỤC vs NHÓM MENU</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>Danh mục</v>
+      </c>
+      <c r="B20" t="str">
+        <v>Dùng để khách lọc món trên trang chủ app (Bún-Phở, Cơm, Cà phê...) — chọn từ dropdown</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>Nhóm menu</v>
+      </c>
+      <c r="B21" t="str">
+        <v>Dùng để nhóm món trong trang quán (Cà phê, Trà sữa, Cơm trưa...) — tự điền tên</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>📌 LOGIC GHÉP DANH MỤC</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v/>
+      </c>
+      <c r="B24" t="str">
+        <v>Danh mục 1, 2, 3 tự động bỏ trùng và bỏ trống khi lưu</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v/>
+      </c>
+      <c r="B25" t="str">
+        <v>VD: Cat1=Cà phê - Trà sữa | Cat2=Cà phê - Trà sữa | Cat3=Ăn vặt - Vỉa hè</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v/>
+      </c>
+      <c r="B26" t="str">
+        <v>→ Kết quả lưu: Cà phê - Trà sữa, Ăn vặt - Vỉa hè</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:B26"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:A12"/>
+  <cols>
+    <col min="1" max="1" width="24.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Bún - Phở - Mì</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Cơm - Cơm hộp</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Cà phê - Trà sữa</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Gà rán - FastFood</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Bánh mì - Sandwich</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Ăn vặt - Vỉa hè</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>🔶 BƯỚC 3</v>
-      </c>
-      <c r="B7" t="str">
-        <v>Lưu file → Vào Admin App → Quản lý → Import Menu → chọn file này</v>
+        <v>Nhậu - Bia hơi</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>🔶 BƯỚC 4</v>
-      </c>
-      <c r="B8" t="str">
-        <v>Hệ thống tự tìm quán theo SĐT → xem preview → bấm Lưu</v>
+        <v>Chay - Healthy</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>Lẩu - Nướng - BBQ</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>📌 MÔ TẢ CỘT</v>
-      </c>
-      <c r="B10" t="str">
-        <v/>
+        <v>Bánh - Tráng miệng</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>Cột A</v>
-      </c>
-      <c r="B11" t="str">
-        <v>Danh mục ứng dụng (tối đa 3, cách nhau bằng dấu phẩy): Nước uống, Buổi sáng, Cơm...</v>
+        <v>Hải sản - Đặc sản</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>Cột B</v>
-      </c>
-      <c r="B12" t="str">
-        <v>Nhóm menu hiển thị trong trang quán: Cà phê, Trà sữa, Cơm...</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="str">
-        <v>Cột C ★</v>
-      </c>
-      <c r="B13" t="str">
-        <v>Tên món (bắt buộc)</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="str">
-        <v>Cột D</v>
-      </c>
-      <c r="B14" t="str">
-        <v>Mô tả / Nguyên liệu</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="str">
-        <v>Cột E ★</v>
-      </c>
-      <c r="B15" t="str">
-        <v>Giá bán (số nguyên VNĐ, bắt buộc)</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="str">
-        <v>Cột F</v>
-      </c>
-      <c r="B16" t="str">
-        <v>Giá khuyến mãi (để trống nếu không có)</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="str">
-        <v>Cột G</v>
-      </c>
-      <c r="B17" t="str">
-        <v>Badge: hot / bigsale / bestseller / new</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="str">
-        <v>Cột H</v>
-      </c>
-      <c r="B18" t="str">
-        <v>Đang bán: CÓ hoặc KHÔNG</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="str">
-        <v>Cột I</v>
-      </c>
-      <c r="B19" t="str">
-        <v>Giờ bán từ (VD: 07:00)</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="str">
-        <v>Cột J</v>
-      </c>
-      <c r="B20" t="str">
-        <v>Giờ bán đến (VD: 22:00)</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="str">
-        <v>Cột K</v>
-      </c>
-      <c r="B21" t="str">
-        <v>Sizes (VD: Nhỏ:15000,Vừa:20000,Lớn:25000)</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="str">
-        <v>Cột L</v>
-      </c>
-      <c r="B22" t="str">
-        <v>Toppings (VD: Trân châu:5000;Thạch:5000)</v>
+        <v>Khác</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B22"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:A12"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix(template): chữ đen nền trắng ở dòng mẫu
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/template_nhap_menu_giao_nhanh.xlsx
+++ b/public/template_nhap_menu_giao_nhanh.xlsx
@@ -210,7 +210,7 @@
       <name val="Arial"/>
     </font>
     <font>
-      <color rgb="FFFFFFFF"/>
+      <color rgb="FF000000"/>
       <sz val="9"/>
       <name val="Arial"/>
     </font>
@@ -240,7 +240,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF1A1208"/>
+        <fgColor rgb="FFFFFFFF"/>
       </patternFill>
     </fill>
   </fills>

</xml_diff>